<commit_message>
refactor: utilise directement le DataType profile EU AccessionNumberIdentifierEuImaging
Le profil HL7 Europe est désormais publié (hl7.fhir.eu.imaging 1.0.0-ballot,
FHIR R4) : supprime le wrapper FRCoreAccessionNumberIdentifierProfile, qui
n'était qu'une solution transitoire, et référence le profil EU directement
sur ServiceRequest.identifier[accessionNumber].

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com> 8fbd230464184b1ac7ba3e64a9cbdf2885f4ea15
</commit_message>
<xml_diff>
--- a/nr-doc-core-service-request/ig/StructureDefinition-fr-core-service-request.xlsx
+++ b/nr-doc-core-service-request/ig/StructureDefinition-fr-core-service-request.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-16T07:37:42+00:00</t>
+    <t>2026-09-17T12:36:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -543,7 +543,7 @@
     <t>accessionNumber</t>
   </si>
   <si>
-    <t xml:space="preserve">Identifier {https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-accession-number-identifier|2.2.0}
+    <t xml:space="preserve">Identifier {http://hl7.eu/fhir/imaging/StructureDefinition/AccessionNumberIdentifierEuImaging|1.0.0-ballot}
 </t>
   </si>
   <si>

</xml_diff>